<commit_message>
Elv: PCA ref site
</commit_message>
<xml_diff>
--- a/res/tabela de habitat.xlsx
+++ b/res/tabela de habitat.xlsx
@@ -1,27 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/480d9b848b88e342/MSS/_Zoo-Rebio/ZooRebio3-23_24/rebio23-part/res/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="11_B992312702E16491F0173ED363DF1AC8AA5AB716" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F937B91F-B74B-4153-A5AE-ECC7D158DEBE}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-22425" windowWidth="21840" windowHeight="37920" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-22425" windowWidth="21840" windowHeight="37920" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
-    <sheet name="tabela_final" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet 1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="tabela_final" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="672" uniqueCount="250">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="500" uniqueCount="500">
   <si>
     <t>Variable</t>
   </si>
@@ -771,13 +764,764 @@
   </si>
   <si>
     <t>17.5 (5-25)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Variable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ponto5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ponto6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ponto7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ponto8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ponto9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ponto10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ponto12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ponto13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ponto14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ponto15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ponto16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ponto17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ponto18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ponto19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ponto20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">w.Cond.uS.cm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">137.5 (119.2-164.4)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">148 (134.1-156.8)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">137.5 (98.3-160.2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">154.2 (141.6-161.8)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">148.2 (120.8-165.5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">140.7 (105-157.9)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">111.7 (85.2-129.8)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">98.8 (78.3-122.4)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">139.4 (92.2-184.2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">223 (172.5-250.8)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">153.5 (109.3-212.5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">123.4 (110.9-130.6)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">121.1 (100.8-136.6)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">130.9 (123.7-139.7)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">134.2 (125.6-139.6)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">w.Turb.ntu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5 (2-10.7)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.9 (2.1-14.1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.9 (1.5-9.2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.7 (4-6.8)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15.1 (11-17.7)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21.5 (10-34.8)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">79.2 (2-346)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11.7 (2-21)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">27.8 (7-44)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11.7 (6-21)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11.3 (5-20)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">32 (11.9-61)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">30.1 (9.3-64)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.2 (4.3-14)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11.2 (8-14.2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">w.pH</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.9 (4.7-7.5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.7 (4.6-7.7)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.1 (4.5-6)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.5 (5-6)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6 (5.3-6.6)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6.1 (5.3-7.3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.8 (5.3-6.4)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.9 (5.5-6.2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6.1 (6-6.5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6.3 (6-6.6)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6.5 (6.2-6.9)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6.4 (6.3-6.6)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6.5 (6-6.8)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6.7 (6.4-7)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6.9 (6.7-7.4)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">m.Elev.m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">107.1 (107.1-107.1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">112.8 (112.8-112.8)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">89 (89-89)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">89.1 (89.1-89.1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">71 (71-71)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">41.5 (41.5-41.5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">80 (80-80)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">87 (87-87)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">76 (76-76)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">86 (86-86)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">49 (49-49)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">47 (47-47)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">54 (54-54)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">m.Vel.m.s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.073 (0.025-0.161)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.086 (0.035-0.24)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.135 (0.022-0.207)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.036 (0-0.115)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.261 (0.172-0.348)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.04 (0-0.119)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.271 (0.055-0.588)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.254 (0.021-0.423)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.296 (0.047-0.461)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.195 (0.09-0.302)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0 (0-0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.272 (0.084-0.508)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.118 (0.054-0.182)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.41 (0.33-0.557)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.22 (0.115-0.37)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">m.Slope</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.4 (1-2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.7 (2.5-3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.4 (1.5-3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.5 (1-2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.1 (1.5-3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.2 (1-2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.3 (1-2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.8 (1-2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.2 (2.5-3.5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.3 (1.5-2.5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 (1-1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.1 (1-3.5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.4 (2-3.5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.9 (1.5-3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">m.Depth.avg.cm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12.8 (9-14)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23.7 (16.3-31.7)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23.8 (16-41)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">43.3 (28.3-51.3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22.1 (15-29)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">35.2 (25.3-40.7)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13.2 (5.3-22.7)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22.6 (10.3-36.3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19.8 (10.7-40.7)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">17.2 (10.7-26)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">33 (14-42)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">54.4 (15.7-98.7)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">49.9 (18-65)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">46.2 (34.7-64)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">72.4 (43-110)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">m.Depth.mar.cm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11.8 (3-16)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21.7 (8-30)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18.8 (7-42)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">48.3 (16-87)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18.8 (11-30)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">33.5 (17-52)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.7 (6-15)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19.5 (11-38)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12.7 (10-15)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13.7 (8-23)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20.3 (12-33)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">38.3 (5-100)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">28.8 (9-50)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">41.5 (28-57)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">49 (20-94)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">s.Mud</t>
+  </si>
+  <si>
+    <t xml:space="preserve">100 (100-100)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">95 (90-100)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">74.2 (5-100)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">38.3 (5-80)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">36.7 (10-100)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">90 (90-90)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">61.7 (10-90)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7.5 (0-30)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7.5 (0-10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">83.3 (0-100)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">97.5 (90-100)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">68.3 (5-100)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.7 (0-5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">66.7 (5-100)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">s.Sand</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5 (0-10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">25.8 (0-95)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">61.7 (20-95)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">63.3 (0-90)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10 (10-10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">38.3 (10-90)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">91.7 (70-100)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">90.8 (80-100)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16.7 (0-100)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.8 (0-5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">30 (0-95)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">98.3 (95-100)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">33.3 (0-95)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">s.Gravel.f</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.7 (0-10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">s.Rocks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">h.Macrophytes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.8 (5-10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10 (0-30)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">17.9 (0-60)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20.8 (0-50)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.2 (0-15)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">h.Algae</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.5 (0-5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.2 (0-1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.5 (0-21)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19.2 (15-25)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">h.Subm.veg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7.5 (5-15)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8.3 (5-15)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.8 (0-10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.8 (0-20)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6.7 (0-15)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5 (0-15)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16.7 (5-20)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10 (5-15)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10 (0-20)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8.3 (0-25)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">h.Overh.veg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">68.3 (40-90)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">70.8 (50-85)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">76.7 (60-90)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">31.7 (25-50)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">70 (60-80)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5 (0-20)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">83.3 (75-90)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">63.3 (30-80)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">65.8 (50-85)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">50 (40-70)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20.8 (10-30)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">33.3 (0-70)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">61.7 (50-70)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">61.7 (40-80)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">h.Grass</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.3 (0-10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6 (0-15)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">27.1 (15-50)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21.8 (1-50)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">39.2 (15-50)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.2 (0-10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">h.Leaf.l</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7.5 (5-10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11 (1-25)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15.8 (5-30)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18.3 (10-30)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.2 (1-30)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.5 (0-10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6.7 (5-10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5 (5-5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.2 (0-5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8.3 (0-15)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">h.Root.masses</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.8 (5-15)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12.5 (5-20)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">42.5 (5-90)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11.7 (5-20)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9.2 (0-25)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.8 (0-15)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11.7 (10-15)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">h.Debris</t>
+  </si>
+  <si>
+    <t xml:space="preserve">30.8 (20-45)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12.7 (5-20)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">17.7 (5-30)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21.7 (5-35)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16.8 (1-40)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8.3 (0-20)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22.2 (8-40)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">25.8 (10-40)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23.3 (10-30)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18.3 (10-40)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">25.8 (0-45)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20 (0-35)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">17.5 (5-25)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="0"/>
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -1103,1058 +1847,1058 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P21"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="1">
       <c r="A1" t="s">
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
+        <v>251</v>
       </c>
       <c r="C1" t="s">
-        <v>2</v>
+        <v>252</v>
       </c>
       <c r="D1" t="s">
-        <v>3</v>
+        <v>253</v>
       </c>
       <c r="E1" t="s">
-        <v>4</v>
+        <v>254</v>
       </c>
       <c r="F1" t="s">
-        <v>5</v>
+        <v>255</v>
       </c>
       <c r="G1" t="s">
-        <v>6</v>
+        <v>256</v>
       </c>
       <c r="H1" t="s">
-        <v>7</v>
+        <v>257</v>
       </c>
       <c r="I1" t="s">
-        <v>8</v>
+        <v>258</v>
       </c>
       <c r="J1" t="s">
-        <v>9</v>
+        <v>259</v>
       </c>
       <c r="K1" t="s">
-        <v>10</v>
+        <v>260</v>
       </c>
       <c r="L1" t="s">
-        <v>11</v>
+        <v>261</v>
       </c>
       <c r="M1" t="s">
-        <v>12</v>
+        <v>262</v>
       </c>
       <c r="N1" t="s">
-        <v>13</v>
+        <v>263</v>
       </c>
       <c r="O1" t="s">
-        <v>14</v>
+        <v>264</v>
       </c>
       <c r="P1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" t="s">
-        <v>16</v>
+        <v>266</v>
       </c>
       <c r="B2" t="s">
-        <v>17</v>
+        <v>267</v>
       </c>
       <c r="C2" t="s">
-        <v>18</v>
+        <v>268</v>
       </c>
       <c r="D2" t="s">
-        <v>19</v>
+        <v>269</v>
       </c>
       <c r="E2" t="s">
-        <v>20</v>
+        <v>270</v>
       </c>
       <c r="F2" t="s">
-        <v>21</v>
+        <v>271</v>
       </c>
       <c r="G2" t="s">
-        <v>22</v>
+        <v>272</v>
       </c>
       <c r="H2" t="s">
-        <v>23</v>
+        <v>273</v>
       </c>
       <c r="I2" t="s">
-        <v>24</v>
+        <v>274</v>
       </c>
       <c r="J2" t="s">
-        <v>25</v>
+        <v>275</v>
       </c>
       <c r="K2" t="s">
-        <v>26</v>
+        <v>276</v>
       </c>
       <c r="L2" t="s">
-        <v>27</v>
+        <v>277</v>
       </c>
       <c r="M2" t="s">
-        <v>28</v>
+        <v>278</v>
       </c>
       <c r="N2" t="s">
-        <v>29</v>
+        <v>279</v>
       </c>
       <c r="O2" t="s">
-        <v>30</v>
+        <v>280</v>
       </c>
       <c r="P2" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="3">
       <c r="A3" t="s">
-        <v>32</v>
+        <v>282</v>
       </c>
       <c r="B3" t="s">
-        <v>33</v>
+        <v>283</v>
       </c>
       <c r="C3" t="s">
-        <v>34</v>
+        <v>284</v>
       </c>
       <c r="D3" t="s">
-        <v>35</v>
+        <v>285</v>
       </c>
       <c r="E3" t="s">
-        <v>36</v>
+        <v>286</v>
       </c>
       <c r="F3" t="s">
-        <v>37</v>
+        <v>287</v>
       </c>
       <c r="G3" t="s">
-        <v>38</v>
+        <v>288</v>
       </c>
       <c r="H3" t="s">
-        <v>39</v>
+        <v>289</v>
       </c>
       <c r="I3" t="s">
-        <v>40</v>
+        <v>290</v>
       </c>
       <c r="J3" t="s">
-        <v>41</v>
+        <v>291</v>
       </c>
       <c r="K3" t="s">
-        <v>42</v>
+        <v>292</v>
       </c>
       <c r="L3" t="s">
-        <v>43</v>
+        <v>293</v>
       </c>
       <c r="M3" t="s">
-        <v>44</v>
+        <v>294</v>
       </c>
       <c r="N3" t="s">
-        <v>45</v>
+        <v>295</v>
       </c>
       <c r="O3" t="s">
-        <v>46</v>
+        <v>296</v>
       </c>
       <c r="P3" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="4">
       <c r="A4" t="s">
-        <v>48</v>
+        <v>298</v>
       </c>
       <c r="B4" t="s">
-        <v>49</v>
+        <v>299</v>
       </c>
       <c r="C4" t="s">
-        <v>50</v>
+        <v>300</v>
       </c>
       <c r="D4" t="s">
-        <v>51</v>
+        <v>301</v>
       </c>
       <c r="E4" t="s">
-        <v>52</v>
+        <v>302</v>
       </c>
       <c r="F4" t="s">
-        <v>53</v>
+        <v>303</v>
       </c>
       <c r="G4" t="s">
-        <v>54</v>
+        <v>304</v>
       </c>
       <c r="H4" t="s">
-        <v>55</v>
+        <v>305</v>
       </c>
       <c r="I4" t="s">
-        <v>56</v>
+        <v>306</v>
       </c>
       <c r="J4" t="s">
-        <v>57</v>
+        <v>307</v>
       </c>
       <c r="K4" t="s">
-        <v>58</v>
+        <v>308</v>
       </c>
       <c r="L4" t="s">
-        <v>59</v>
+        <v>309</v>
       </c>
       <c r="M4" t="s">
-        <v>60</v>
+        <v>310</v>
       </c>
       <c r="N4" t="s">
-        <v>61</v>
+        <v>311</v>
       </c>
       <c r="O4" t="s">
-        <v>62</v>
+        <v>312</v>
       </c>
       <c r="P4" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="5">
       <c r="A5" t="s">
-        <v>64</v>
+        <v>314</v>
       </c>
       <c r="B5" t="s">
-        <v>65</v>
+        <v>315</v>
       </c>
       <c r="C5" t="s">
-        <v>66</v>
+        <v>316</v>
       </c>
       <c r="D5" t="s">
-        <v>67</v>
+        <v>317</v>
       </c>
       <c r="E5" t="s">
-        <v>68</v>
+        <v>318</v>
       </c>
       <c r="F5" t="s">
-        <v>69</v>
+        <v>319</v>
       </c>
       <c r="G5" t="s">
-        <v>70</v>
+        <v>320</v>
       </c>
       <c r="H5" t="s">
-        <v>71</v>
+        <v>321</v>
       </c>
       <c r="I5" t="s">
-        <v>72</v>
+        <v>322</v>
       </c>
       <c r="J5" t="s">
-        <v>73</v>
+        <v>323</v>
       </c>
       <c r="K5" t="s">
-        <v>74</v>
+        <v>324</v>
       </c>
       <c r="L5" t="s">
-        <v>73</v>
+        <v>323</v>
       </c>
       <c r="M5" t="s">
-        <v>75</v>
+        <v>325</v>
       </c>
       <c r="N5" t="s">
-        <v>76</v>
+        <v>326</v>
       </c>
       <c r="O5" t="s">
-        <v>77</v>
+        <v>327</v>
       </c>
       <c r="P5" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="6">
       <c r="A6" t="s">
-        <v>78</v>
+        <v>328</v>
       </c>
       <c r="B6" t="s">
-        <v>79</v>
+        <v>329</v>
       </c>
       <c r="C6" t="s">
-        <v>80</v>
+        <v>330</v>
       </c>
       <c r="D6" t="s">
-        <v>81</v>
+        <v>331</v>
       </c>
       <c r="E6" t="s">
-        <v>82</v>
+        <v>332</v>
       </c>
       <c r="F6" t="s">
-        <v>83</v>
+        <v>333</v>
       </c>
       <c r="G6" t="s">
-        <v>84</v>
+        <v>334</v>
       </c>
       <c r="H6" t="s">
-        <v>85</v>
+        <v>335</v>
       </c>
       <c r="I6" t="s">
-        <v>86</v>
+        <v>336</v>
       </c>
       <c r="J6" t="s">
-        <v>87</v>
+        <v>337</v>
       </c>
       <c r="K6" t="s">
-        <v>88</v>
+        <v>338</v>
       </c>
       <c r="L6" t="s">
-        <v>89</v>
+        <v>339</v>
       </c>
       <c r="M6" t="s">
-        <v>90</v>
+        <v>340</v>
       </c>
       <c r="N6" t="s">
-        <v>91</v>
+        <v>341</v>
       </c>
       <c r="O6" t="s">
-        <v>92</v>
+        <v>342</v>
       </c>
       <c r="P6" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="7">
       <c r="A7" t="s">
-        <v>94</v>
+        <v>344</v>
       </c>
       <c r="B7" t="s">
-        <v>95</v>
+        <v>345</v>
       </c>
       <c r="C7" t="s">
-        <v>96</v>
+        <v>346</v>
       </c>
       <c r="D7" t="s">
-        <v>97</v>
+        <v>347</v>
       </c>
       <c r="E7" t="s">
-        <v>98</v>
+        <v>348</v>
       </c>
       <c r="F7" t="s">
-        <v>99</v>
+        <v>349</v>
       </c>
       <c r="G7" t="s">
-        <v>100</v>
+        <v>350</v>
       </c>
       <c r="H7" t="s">
-        <v>101</v>
+        <v>351</v>
       </c>
       <c r="I7" t="s">
-        <v>102</v>
+        <v>352</v>
       </c>
       <c r="J7" t="s">
-        <v>103</v>
+        <v>353</v>
       </c>
       <c r="K7" t="s">
-        <v>104</v>
+        <v>354</v>
       </c>
       <c r="L7" t="s">
-        <v>105</v>
+        <v>355</v>
       </c>
       <c r="M7" t="s">
-        <v>106</v>
+        <v>356</v>
       </c>
       <c r="N7" t="s">
-        <v>105</v>
+        <v>355</v>
       </c>
       <c r="O7" t="s">
-        <v>107</v>
+        <v>357</v>
       </c>
       <c r="P7" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="8">
       <c r="A8" t="s">
-        <v>109</v>
+        <v>359</v>
       </c>
       <c r="B8" t="s">
-        <v>110</v>
+        <v>360</v>
       </c>
       <c r="C8" t="s">
-        <v>111</v>
+        <v>361</v>
       </c>
       <c r="D8" t="s">
-        <v>112</v>
+        <v>362</v>
       </c>
       <c r="E8" t="s">
-        <v>113</v>
+        <v>363</v>
       </c>
       <c r="F8" t="s">
-        <v>114</v>
+        <v>364</v>
       </c>
       <c r="G8" t="s">
-        <v>115</v>
+        <v>365</v>
       </c>
       <c r="H8" t="s">
-        <v>116</v>
+        <v>366</v>
       </c>
       <c r="I8" t="s">
-        <v>117</v>
+        <v>367</v>
       </c>
       <c r="J8" t="s">
-        <v>118</v>
+        <v>368</v>
       </c>
       <c r="K8" t="s">
-        <v>119</v>
+        <v>369</v>
       </c>
       <c r="L8" t="s">
-        <v>120</v>
+        <v>370</v>
       </c>
       <c r="M8" t="s">
-        <v>121</v>
+        <v>371</v>
       </c>
       <c r="N8" t="s">
-        <v>122</v>
+        <v>372</v>
       </c>
       <c r="O8" t="s">
-        <v>123</v>
+        <v>373</v>
       </c>
       <c r="P8" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="9">
       <c r="A9" t="s">
-        <v>125</v>
+        <v>375</v>
       </c>
       <c r="B9" t="s">
-        <v>126</v>
+        <v>376</v>
       </c>
       <c r="C9" t="s">
-        <v>127</v>
+        <v>377</v>
       </c>
       <c r="D9" t="s">
-        <v>128</v>
+        <v>378</v>
       </c>
       <c r="E9" t="s">
-        <v>129</v>
+        <v>379</v>
       </c>
       <c r="F9" t="s">
-        <v>130</v>
+        <v>380</v>
       </c>
       <c r="G9" t="s">
-        <v>131</v>
+        <v>381</v>
       </c>
       <c r="H9" t="s">
-        <v>132</v>
+        <v>382</v>
       </c>
       <c r="I9" t="s">
-        <v>133</v>
+        <v>383</v>
       </c>
       <c r="J9" t="s">
-        <v>134</v>
+        <v>384</v>
       </c>
       <c r="K9" t="s">
-        <v>135</v>
+        <v>385</v>
       </c>
       <c r="L9" t="s">
-        <v>136</v>
+        <v>386</v>
       </c>
       <c r="M9" t="s">
-        <v>137</v>
+        <v>387</v>
       </c>
       <c r="N9" t="s">
-        <v>138</v>
+        <v>388</v>
       </c>
       <c r="O9" t="s">
-        <v>139</v>
+        <v>389</v>
       </c>
       <c r="P9" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="10">
       <c r="A10" t="s">
-        <v>141</v>
+        <v>391</v>
       </c>
       <c r="B10" t="s">
-        <v>142</v>
+        <v>392</v>
       </c>
       <c r="C10" t="s">
-        <v>142</v>
+        <v>392</v>
       </c>
       <c r="D10" t="s">
-        <v>143</v>
+        <v>393</v>
       </c>
       <c r="E10" t="s">
-        <v>144</v>
+        <v>394</v>
       </c>
       <c r="F10" t="s">
-        <v>145</v>
+        <v>395</v>
       </c>
       <c r="G10" t="s">
-        <v>146</v>
+        <v>396</v>
       </c>
       <c r="H10" t="s">
-        <v>147</v>
+        <v>397</v>
       </c>
       <c r="I10" t="s">
-        <v>148</v>
+        <v>398</v>
       </c>
       <c r="J10" t="s">
-        <v>149</v>
+        <v>399</v>
       </c>
       <c r="K10" t="s">
-        <v>150</v>
+        <v>400</v>
       </c>
       <c r="L10" t="s">
-        <v>151</v>
+        <v>401</v>
       </c>
       <c r="M10" t="s">
-        <v>152</v>
+        <v>402</v>
       </c>
       <c r="N10" t="s">
-        <v>153</v>
+        <v>403</v>
       </c>
       <c r="O10" t="s">
-        <v>154</v>
+        <v>404</v>
       </c>
       <c r="P10" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="11">
       <c r="A11" t="s">
-        <v>156</v>
+        <v>406</v>
       </c>
       <c r="B11" t="s">
-        <v>89</v>
+        <v>339</v>
       </c>
       <c r="C11" t="s">
-        <v>89</v>
+        <v>339</v>
       </c>
       <c r="D11" t="s">
-        <v>157</v>
+        <v>407</v>
       </c>
       <c r="E11" t="s">
-        <v>158</v>
+        <v>408</v>
       </c>
       <c r="F11" t="s">
-        <v>159</v>
+        <v>409</v>
       </c>
       <c r="G11" t="s">
-        <v>160</v>
+        <v>410</v>
       </c>
       <c r="H11" t="s">
-        <v>161</v>
+        <v>411</v>
       </c>
       <c r="I11" t="s">
-        <v>162</v>
+        <v>412</v>
       </c>
       <c r="J11" t="s">
-        <v>163</v>
+        <v>413</v>
       </c>
       <c r="K11" t="s">
-        <v>164</v>
+        <v>414</v>
       </c>
       <c r="L11" t="s">
-        <v>165</v>
+        <v>415</v>
       </c>
       <c r="M11" t="s">
-        <v>166</v>
+        <v>416</v>
       </c>
       <c r="N11" t="s">
-        <v>167</v>
+        <v>417</v>
       </c>
       <c r="O11" t="s">
-        <v>168</v>
+        <v>418</v>
       </c>
       <c r="P11" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="12">
       <c r="A12" t="s">
-        <v>170</v>
+        <v>420</v>
       </c>
       <c r="B12" t="s">
-        <v>89</v>
+        <v>339</v>
       </c>
       <c r="C12" t="s">
-        <v>89</v>
+        <v>339</v>
       </c>
       <c r="D12" t="s">
-        <v>89</v>
+        <v>339</v>
       </c>
       <c r="E12" t="s">
-        <v>89</v>
+        <v>339</v>
       </c>
       <c r="F12" t="s">
-        <v>89</v>
+        <v>339</v>
       </c>
       <c r="G12" t="s">
-        <v>89</v>
+        <v>339</v>
       </c>
       <c r="H12" t="s">
-        <v>89</v>
+        <v>339</v>
       </c>
       <c r="I12" t="s">
-        <v>89</v>
+        <v>339</v>
       </c>
       <c r="J12" t="s">
-        <v>166</v>
+        <v>416</v>
       </c>
       <c r="K12" t="s">
-        <v>171</v>
+        <v>421</v>
       </c>
       <c r="L12" t="s">
-        <v>89</v>
+        <v>339</v>
       </c>
       <c r="M12" t="s">
-        <v>89</v>
+        <v>339</v>
       </c>
       <c r="N12" t="s">
-        <v>171</v>
+        <v>421</v>
       </c>
       <c r="O12" t="s">
-        <v>89</v>
+        <v>339</v>
       </c>
       <c r="P12" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="13">
       <c r="A13" t="s">
-        <v>172</v>
+        <v>422</v>
       </c>
       <c r="B13" t="s">
-        <v>89</v>
+        <v>339</v>
       </c>
       <c r="C13" t="s">
-        <v>89</v>
+        <v>339</v>
       </c>
       <c r="D13" t="s">
-        <v>89</v>
+        <v>339</v>
       </c>
       <c r="E13" t="s">
-        <v>89</v>
+        <v>339</v>
       </c>
       <c r="F13" t="s">
-        <v>89</v>
+        <v>339</v>
       </c>
       <c r="G13" t="s">
-        <v>89</v>
+        <v>339</v>
       </c>
       <c r="H13" t="s">
-        <v>89</v>
+        <v>339</v>
       </c>
       <c r="I13" t="s">
-        <v>89</v>
+        <v>339</v>
       </c>
       <c r="J13" t="s">
-        <v>89</v>
+        <v>339</v>
       </c>
       <c r="K13" t="s">
-        <v>89</v>
+        <v>339</v>
       </c>
       <c r="L13" t="s">
-        <v>89</v>
+        <v>339</v>
       </c>
       <c r="M13" t="s">
-        <v>171</v>
+        <v>421</v>
       </c>
       <c r="N13" t="s">
-        <v>89</v>
+        <v>339</v>
       </c>
       <c r="O13" t="s">
-        <v>89</v>
+        <v>339</v>
       </c>
       <c r="P13" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="14">
       <c r="A14" t="s">
-        <v>173</v>
+        <v>423</v>
       </c>
       <c r="B14" t="s">
-        <v>174</v>
+        <v>424</v>
       </c>
       <c r="C14" t="s">
-        <v>175</v>
+        <v>425</v>
       </c>
       <c r="D14" t="s">
-        <v>89</v>
+        <v>339</v>
       </c>
       <c r="E14" t="s">
-        <v>176</v>
+        <v>426</v>
       </c>
       <c r="F14" t="s">
-        <v>89</v>
+        <v>339</v>
       </c>
       <c r="G14" t="s">
-        <v>154</v>
+        <v>404</v>
       </c>
       <c r="H14" t="s">
-        <v>89</v>
+        <v>339</v>
       </c>
       <c r="I14" t="s">
-        <v>166</v>
+        <v>416</v>
       </c>
       <c r="J14" t="s">
-        <v>89</v>
+        <v>339</v>
       </c>
       <c r="K14" t="s">
-        <v>89</v>
+        <v>339</v>
       </c>
       <c r="L14" t="s">
-        <v>177</v>
+        <v>427</v>
       </c>
       <c r="M14" t="s">
-        <v>89</v>
+        <v>339</v>
       </c>
       <c r="N14" t="s">
-        <v>178</v>
+        <v>428</v>
       </c>
       <c r="O14" t="s">
-        <v>89</v>
+        <v>339</v>
       </c>
       <c r="P14" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="15">
       <c r="A15" t="s">
-        <v>179</v>
+        <v>429</v>
       </c>
       <c r="B15" t="s">
-        <v>180</v>
+        <v>430</v>
       </c>
       <c r="C15" t="s">
-        <v>181</v>
+        <v>431</v>
       </c>
       <c r="D15" t="s">
-        <v>182</v>
+        <v>432</v>
       </c>
       <c r="E15" t="s">
-        <v>183</v>
+        <v>433</v>
       </c>
       <c r="F15" t="s">
-        <v>89</v>
+        <v>339</v>
       </c>
       <c r="G15" t="s">
-        <v>184</v>
+        <v>416</v>
       </c>
       <c r="H15" t="s">
-        <v>89</v>
+        <v>416</v>
       </c>
       <c r="I15" t="s">
-        <v>89</v>
+        <v>339</v>
       </c>
       <c r="J15" t="s">
-        <v>89</v>
+        <v>339</v>
       </c>
       <c r="K15" t="s">
-        <v>166</v>
+        <v>339</v>
       </c>
       <c r="L15" t="s">
-        <v>185</v>
+        <v>339</v>
       </c>
       <c r="M15" t="s">
-        <v>174</v>
+        <v>339</v>
       </c>
       <c r="N15" t="s">
-        <v>186</v>
+        <v>339</v>
       </c>
       <c r="O15" t="s">
-        <v>89</v>
+        <v>339</v>
       </c>
       <c r="P15" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="16">
       <c r="A16" t="s">
-        <v>187</v>
+        <v>434</v>
       </c>
       <c r="B16" t="s">
-        <v>188</v>
+        <v>435</v>
       </c>
       <c r="C16" t="s">
-        <v>181</v>
+        <v>436</v>
       </c>
       <c r="D16" t="s">
-        <v>189</v>
+        <v>437</v>
       </c>
       <c r="E16" t="s">
-        <v>189</v>
+        <v>437</v>
       </c>
       <c r="F16" t="s">
-        <v>190</v>
+        <v>438</v>
       </c>
       <c r="G16" t="s">
-        <v>157</v>
+        <v>407</v>
       </c>
       <c r="H16" t="s">
-        <v>154</v>
+        <v>404</v>
       </c>
       <c r="I16" t="s">
-        <v>191</v>
+        <v>439</v>
       </c>
       <c r="J16" t="s">
-        <v>192</v>
+        <v>440</v>
       </c>
       <c r="K16" t="s">
-        <v>89</v>
+        <v>339</v>
       </c>
       <c r="L16" t="s">
-        <v>193</v>
+        <v>441</v>
       </c>
       <c r="M16" t="s">
-        <v>194</v>
+        <v>442</v>
       </c>
       <c r="N16" t="s">
-        <v>195</v>
+        <v>443</v>
       </c>
       <c r="O16" t="s">
-        <v>166</v>
+        <v>416</v>
       </c>
       <c r="P16" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="17">
       <c r="A17" t="s">
-        <v>197</v>
+        <v>445</v>
       </c>
       <c r="B17" t="s">
-        <v>198</v>
+        <v>446</v>
       </c>
       <c r="C17" t="s">
-        <v>199</v>
+        <v>447</v>
       </c>
       <c r="D17" t="s">
-        <v>200</v>
+        <v>448</v>
       </c>
       <c r="E17" t="s">
-        <v>201</v>
+        <v>449</v>
       </c>
       <c r="F17" t="s">
-        <v>202</v>
+        <v>450</v>
       </c>
       <c r="G17" t="s">
-        <v>203</v>
+        <v>451</v>
       </c>
       <c r="H17" t="s">
-        <v>204</v>
+        <v>452</v>
       </c>
       <c r="I17" t="s">
-        <v>205</v>
+        <v>453</v>
       </c>
       <c r="J17" t="s">
-        <v>206</v>
+        <v>454</v>
       </c>
       <c r="K17" t="s">
-        <v>207</v>
+        <v>455</v>
       </c>
       <c r="L17" t="s">
-        <v>166</v>
+        <v>416</v>
       </c>
       <c r="M17" t="s">
-        <v>208</v>
+        <v>456</v>
       </c>
       <c r="N17" t="s">
-        <v>209</v>
+        <v>457</v>
       </c>
       <c r="O17" t="s">
-        <v>210</v>
+        <v>458</v>
       </c>
       <c r="P17" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="18">
       <c r="A18" t="s">
-        <v>212</v>
+        <v>460</v>
       </c>
       <c r="B18" t="s">
-        <v>213</v>
+        <v>461</v>
       </c>
       <c r="C18" t="s">
-        <v>214</v>
+        <v>436</v>
       </c>
       <c r="D18" t="s">
-        <v>215</v>
+        <v>462</v>
       </c>
       <c r="E18" t="s">
-        <v>216</v>
+        <v>463</v>
       </c>
       <c r="F18" t="s">
-        <v>217</v>
+        <v>339</v>
       </c>
       <c r="G18" t="s">
-        <v>218</v>
+        <v>464</v>
       </c>
       <c r="H18" t="s">
-        <v>188</v>
+        <v>339</v>
       </c>
       <c r="I18" t="s">
-        <v>219</v>
+        <v>339</v>
       </c>
       <c r="J18" t="s">
-        <v>220</v>
+        <v>339</v>
       </c>
       <c r="K18" t="s">
-        <v>213</v>
+        <v>416</v>
       </c>
       <c r="L18" t="s">
-        <v>154</v>
+        <v>465</v>
       </c>
       <c r="M18" t="s">
-        <v>221</v>
+        <v>424</v>
       </c>
       <c r="N18" t="s">
-        <v>157</v>
+        <v>466</v>
       </c>
       <c r="O18" t="s">
-        <v>222</v>
+        <v>339</v>
       </c>
       <c r="P18" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="19">
       <c r="A19" t="s">
-        <v>224</v>
+        <v>467</v>
       </c>
       <c r="B19" t="s">
-        <v>192</v>
+        <v>468</v>
       </c>
       <c r="C19" t="s">
-        <v>225</v>
+        <v>469</v>
       </c>
       <c r="D19" t="s">
-        <v>226</v>
+        <v>470</v>
       </c>
       <c r="E19" t="s">
-        <v>186</v>
+        <v>471</v>
       </c>
       <c r="F19" t="s">
-        <v>227</v>
+        <v>472</v>
       </c>
       <c r="G19" t="s">
-        <v>180</v>
+        <v>473</v>
       </c>
       <c r="H19" t="s">
-        <v>189</v>
+        <v>435</v>
       </c>
       <c r="I19" t="s">
-        <v>194</v>
+        <v>474</v>
       </c>
       <c r="J19" t="s">
-        <v>228</v>
+        <v>475</v>
       </c>
       <c r="K19" t="s">
-        <v>229</v>
+        <v>468</v>
       </c>
       <c r="L19" t="s">
-        <v>166</v>
+        <v>404</v>
       </c>
       <c r="M19" t="s">
-        <v>225</v>
+        <v>430</v>
       </c>
       <c r="N19" t="s">
-        <v>230</v>
+        <v>407</v>
       </c>
       <c r="O19" t="s">
-        <v>188</v>
+        <v>476</v>
       </c>
       <c r="P19" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="20">
       <c r="A20" t="s">
-        <v>232</v>
+        <v>478</v>
       </c>
       <c r="B20" t="s">
-        <v>221</v>
+        <v>440</v>
       </c>
       <c r="C20" t="s">
-        <v>233</v>
+        <v>479</v>
       </c>
       <c r="D20" t="s">
-        <v>234</v>
+        <v>480</v>
       </c>
       <c r="E20" t="s">
-        <v>235</v>
+        <v>466</v>
       </c>
       <c r="F20" t="s">
-        <v>89</v>
+        <v>481</v>
       </c>
       <c r="G20" t="s">
-        <v>166</v>
+        <v>461</v>
       </c>
       <c r="H20" t="s">
-        <v>166</v>
+        <v>437</v>
       </c>
       <c r="I20" t="s">
-        <v>89</v>
+        <v>442</v>
       </c>
       <c r="J20" t="s">
-        <v>89</v>
+        <v>482</v>
       </c>
       <c r="K20" t="s">
-        <v>89</v>
+        <v>483</v>
       </c>
       <c r="L20" t="s">
-        <v>89</v>
+        <v>416</v>
       </c>
       <c r="M20" t="s">
-        <v>89</v>
+        <v>479</v>
       </c>
       <c r="N20" t="s">
-        <v>89</v>
+        <v>484</v>
       </c>
       <c r="O20" t="s">
-        <v>89</v>
+        <v>435</v>
       </c>
       <c r="P20" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="21">
       <c r="A21" t="s">
-        <v>236</v>
+        <v>486</v>
       </c>
       <c r="B21" t="s">
-        <v>237</v>
+        <v>487</v>
       </c>
       <c r="C21" t="s">
-        <v>238</v>
+        <v>488</v>
       </c>
       <c r="D21" t="s">
-        <v>239</v>
+        <v>489</v>
       </c>
       <c r="E21" t="s">
-        <v>240</v>
+        <v>490</v>
       </c>
       <c r="F21" t="s">
-        <v>241</v>
+        <v>491</v>
       </c>
       <c r="G21" t="s">
-        <v>242</v>
+        <v>492</v>
       </c>
       <c r="H21" t="s">
-        <v>243</v>
+        <v>493</v>
       </c>
       <c r="I21" t="s">
-        <v>244</v>
+        <v>494</v>
       </c>
       <c r="J21" t="s">
-        <v>245</v>
+        <v>495</v>
       </c>
       <c r="K21" t="s">
-        <v>246</v>
+        <v>496</v>
       </c>
       <c r="L21" t="s">
-        <v>186</v>
+        <v>466</v>
       </c>
       <c r="M21" t="s">
-        <v>247</v>
+        <v>497</v>
       </c>
       <c r="N21" t="s">
-        <v>248</v>
+        <v>498</v>
       </c>
       <c r="O21" t="s">
-        <v>178</v>
+        <v>428</v>
       </c>
       <c r="P21" t="s">
-        <v>249</v>
+        <v>499</v>
       </c>
     </row>
   </sheetData>
@@ -2164,11 +2908,11 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F72FDC22-1824-479A-BC36-CF8D433CAFCA}">
-  <dimension ref="A1:P21"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="1">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2218,7 +2962,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="2">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -2268,7 +3012,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="3">
       <c r="A3" t="s">
         <v>32</v>
       </c>
@@ -2318,7 +3062,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="4">
       <c r="A4" t="s">
         <v>48</v>
       </c>
@@ -2368,7 +3112,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="5">
       <c r="A5" t="s">
         <v>64</v>
       </c>
@@ -2418,7 +3162,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="6">
       <c r="A6" t="s">
         <v>78</v>
       </c>
@@ -2468,7 +3212,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="7">
       <c r="A7" t="s">
         <v>94</v>
       </c>
@@ -2518,7 +3262,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="8">
       <c r="A8" t="s">
         <v>109</v>
       </c>
@@ -2568,7 +3312,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="9">
       <c r="A9" t="s">
         <v>125</v>
       </c>
@@ -2618,7 +3362,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="10">
       <c r="A10" t="s">
         <v>141</v>
       </c>
@@ -2668,7 +3412,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="11">
       <c r="A11" t="s">
         <v>156</v>
       </c>
@@ -2718,7 +3462,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="12">
       <c r="A12" t="s">
         <v>170</v>
       </c>
@@ -2768,7 +3512,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="13">
       <c r="A13" t="s">
         <v>172</v>
       </c>
@@ -2818,7 +3562,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="14">
       <c r="A14" t="s">
         <v>173</v>
       </c>
@@ -2868,7 +3612,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="15">
       <c r="A15" t="s">
         <v>179</v>
       </c>
@@ -2918,7 +3662,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="16">
       <c r="A16" t="s">
         <v>187</v>
       </c>
@@ -2968,7 +3712,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="17">
       <c r="A17" t="s">
         <v>197</v>
       </c>
@@ -3018,7 +3762,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="18">
       <c r="A18" t="s">
         <v>212</v>
       </c>
@@ -3068,7 +3812,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="19">
       <c r="A19" t="s">
         <v>224</v>
       </c>
@@ -3118,7 +3862,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="20">
       <c r="A20" t="s">
         <v>232</v>
       </c>
@@ -3168,7 +3912,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="21">
       <c r="A21" t="s">
         <v>236</v>
       </c>
@@ -3220,5 +3964,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>